<commit_message>
Finaliza integração Google Drive na página de Configurações
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentos/resources/diario_bordo.xlsx
+++ b/documentos/resources/diario_bordo.xlsx
@@ -109,7 +109,7 @@
     <t xml:space="preserve">NOME: {{motorista}}</t>
   </si>
   <si>
-    <t xml:space="preserve">RG: {{rg_motorista}}</t>
+    <t xml:space="preserve">CPF: {{cpf_motorista}}</t>
   </si>
   <si>
     <t xml:space="preserve">ASSINATURA:</t>
@@ -242,36 +242,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -298,9 +302,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>357840</xdr:colOff>
+      <xdr:colOff>357480</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>66240</xdr:rowOff>
+      <xdr:rowOff>65880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -314,7 +318,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7223760" y="0"/>
-          <a:ext cx="799920" cy="1095120"/>
+          <a:ext cx="799560" cy="1094760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -511,354 +515,354 @@
   <dimension ref="A1:L20"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="1" style="0" width="18.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="1" style="1" width="18.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5" t="s">
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5" t="s">
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5" t="s">
+      <c r="H15" s="6"/>
+      <c r="I15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5" t="s">
+      <c r="J15" s="6"/>
+      <c r="K15" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="L15" s="5"/>
+      <c r="L15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="6"/>
-      <c r="I17" s="7" t="s">
+      <c r="H17" s="7"/>
+      <c r="I17" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="J17" s="7"/>
-      <c r="K17" s="6" t="s">
+      <c r="J17" s="8"/>
+      <c r="K17" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="L17" s="6"/>
+      <c r="L17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3" t="s">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3" t="s">
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="23">

</xml_diff>